<commit_message>
feat: Convex migration complete — chat, calls, media, status, settings
- Migrated entire backend from Supabase/Express to Convex
- Real-time chat with message delivery/read receipts
- Voice and video calls via Agora RTC
- Image/video sending with Convex file storage
- Auto-download setting (never/wifi/mobile) with tap-to-load UI
- Full-screen image viewer on tap
- WhatsApp-style chat input: attachment panel, Giphy sticker picker, camera
- Status posts (24h expiry), call history, SOS contacts
- Dark/light theme, font size settings, privacy controls
- Android and iOS native builds added

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/technical/Connex_Project_Tracker.xlsx
+++ b/docs/technical/Connex_Project_Tracker.xlsx
@@ -85,12 +85,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -167,7 +167,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -179,7 +179,7 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Build POST /auth/login endpoint — return JWT + refresh token</t>
+          <t>Build legacy /auth/login bridge for pre-Supabase accounts</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1144,14 +1144,14 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Store refresh token in Redis</t>
+          <t>Migrates older custom-auth users into Supabase Auth</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Build POST /auth/logout — invalidate tokens</t>
+          <t>Verify Supabase access tokens on protected routes</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1186,14 +1186,14 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Delete from Redis</t>
+          <t>Backend auth middleware no longer issues custom JWTs</t>
         </is>
       </c>
     </row>
@@ -1354,14 +1354,14 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Phone OTP via Supabase Auth</t>
+          <t>Direct Supabase sign-up using phone/password UI</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,16 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Direct Supabase login with one-time backend fallback for legacy users</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
@@ -3674,12 +3678,12 @@
           <t>src/screens/auth/OnboardingScreen.tsx</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3711,12 +3715,12 @@
           <t>src/screens/auth/RegisterScreen.tsx</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3748,12 +3752,12 @@
           <t>src/screens/auth/LoginScreen.tsx</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3785,12 +3789,12 @@
           <t>src/screens/auth/ProfileSetupScreen.tsx</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3822,12 +3826,12 @@
           <t>src/screens/chat/ChatListScreen.tsx</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3859,12 +3863,12 @@
           <t>src/screens/chat/ChatRoomScreen.tsx</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3896,12 +3900,12 @@
           <t>src/screens/chat/NewChatScreen.tsx</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3933,12 +3937,12 @@
           <t>src/screens/chat/GroupCreateScreen.tsx</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3970,12 +3974,12 @@
           <t>src/screens/chat/StatusListScreen.tsx</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4007,12 +4011,12 @@
           <t>src/screens/chat/StatusViewScreen.tsx</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4044,12 +4048,12 @@
           <t>src/screens/sos/SOSScreen.tsx</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4081,12 +4085,12 @@
           <t>src/screens/sos/SOSContactsScreen.tsx</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4118,12 +4122,12 @@
           <t>src/screens/feed/FeedHomeScreen.tsx</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4155,12 +4159,12 @@
           <t>src/screens/feed/AlertsTabScreen.tsx</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4192,12 +4196,12 @@
           <t>src/screens/feed/AlertsMapScreen.tsx</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4229,12 +4233,12 @@
           <t>src/screens/feed/CreatePostScreen.tsx</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4266,12 +4270,12 @@
           <t>src/screens/feed/PostDetailScreen.tsx</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4303,12 +4307,12 @@
           <t>src/screens/feed/ExploreScreen.tsx</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4340,12 +4344,12 @@
           <t>src/screens/edu/EduHomeScreen.tsx</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4377,12 +4381,12 @@
           <t>src/screens/edu/PaperListScreen.tsx</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4414,12 +4418,12 @@
           <t>src/screens/edu/PaperViewerScreen.tsx</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4451,12 +4455,12 @@
           <t>src/screens/profile/ProfileScreen.tsx</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4488,12 +4492,12 @@
           <t>src/screens/profile/EditProfileScreen.tsx</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4525,12 +4529,12 @@
           <t>src/screens/profile/SettingsScreen.tsx</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4562,12 +4566,12 @@
           <t>src/screens/NotificationsScreen.tsx</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4599,7 +4603,7 @@
           <t>src/screens/pay/PayHomeScreen.tsx</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4636,7 +4640,7 @@
           <t>src/screens/pay/SendMoneyScreen.tsx</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4673,7 +4677,7 @@
           <t>src/screens/clips/ClipsHomeScreen.tsx</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4710,7 +4714,7 @@
           <t>src/screens/logistics/LogisticsHomeScreen.tsx</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4797,7 +4801,7 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -4817,12 +4821,12 @@
           <t>Register new user (phone, name, password)</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4834,7 +4838,7 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -4851,27 +4855,27 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Login — returns JWT + refresh token</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
+          <t>Legacy-account bridge into Supabase Auth sessions</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Store refresh in Redis</t>
+          <t>Only needed for pre-migration users</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -4888,15 +4892,15 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Logout — invalidate JWT and refresh token</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
+          <t>Revoke current Supabase session from backend if needed</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4904,7 +4908,7 @@
       <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -4921,15 +4925,15 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Refresh JWT using refresh token</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+          <t>Refresh Supabase session using refresh token</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4957,12 +4961,12 @@
           <t>Get user profile by ID</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -4990,12 +4994,12 @@
           <t>Update profile (name, bio, avatar_url)</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5027,12 +5031,12 @@
           <t>Search users by name or phone</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5044,7 +5048,7 @@
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5064,12 +5068,12 @@
           <t>Create new conversation (1:1 or group)</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5097,12 +5101,12 @@
           <t>List all conversations for auth user</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5134,12 +5138,12 @@
           <t>Get single conversation details + members</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5167,12 +5171,12 @@
           <t>Update group name or image</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5184,7 +5188,7 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5204,12 +5208,12 @@
           <t>Add member to group conversation</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5217,7 +5221,7 @@
       <c r="G14" s="4" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
@@ -5237,12 +5241,12 @@
           <t>Remove member from group</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5250,7 +5254,7 @@
       <c r="G15" s="3" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5270,12 +5274,12 @@
           <t>Send a message in a conversation</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5307,12 +5311,12 @@
           <t>Get paginated message history (cursor-based)</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5340,12 +5344,12 @@
           <t>Mark message as read (update status)</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5353,7 +5357,7 @@
       <c r="G18" s="4" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5373,12 +5377,12 @@
           <t>Create post (text, image_url, optional alert_tag)</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5410,12 +5414,12 @@
           <t>Paginated home feed (following + area)</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5447,12 +5451,12 @@
           <t>Get alert posts — filter by tag + area_id</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5484,12 +5488,12 @@
           <t>Get single post with reactions + comments</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5497,7 +5501,7 @@
       <c r="G22" s="4" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
@@ -5517,12 +5521,12 @@
           <t>Delete own post</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5530,7 +5534,7 @@
       <c r="G23" s="3" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5550,12 +5554,12 @@
           <t>Like or react to a post</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5563,7 +5567,7 @@
       <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
@@ -5583,12 +5587,12 @@
           <t>Remove reaction from post</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5596,7 +5600,7 @@
       <c r="G25" s="3" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5616,12 +5620,12 @@
           <t>Follow a user</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5629,7 +5633,7 @@
       <c r="G26" s="4" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
@@ -5649,12 +5653,12 @@
           <t>Unfollow a user</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5682,12 +5686,12 @@
           <t>Get loadshedding schedule for suburb (cached)</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5719,12 +5723,12 @@
           <t>Get current national loadshedding stage</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5736,7 +5740,7 @@
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5756,12 +5760,12 @@
           <t>Add emergency contact (sends accept request)</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5793,12 +5797,12 @@
           <t>List own SOS contacts (pending + accepted)</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5806,7 +5810,7 @@
       <c r="G31" s="3" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5826,12 +5830,12 @@
           <t>Accept incoming SOS contact request</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5839,7 +5843,7 @@
       <c r="G32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
@@ -5859,12 +5863,12 @@
           <t>Remove emergency contact</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5872,7 +5876,7 @@
       <c r="G33" s="3" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5892,12 +5896,12 @@
           <t>Trigger SOS event — notify all accepted contacts</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5909,7 +5913,7 @@
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -5929,12 +5933,12 @@
           <t>Cancel active SOS — notify contacts user is safe</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5962,12 +5966,12 @@
           <t>Get SOS event history</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -5995,12 +5999,12 @@
           <t>Get papers — filter by grade, subject, year</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -6032,12 +6036,12 @@
           <t>Get single paper metadata + download URL</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -6069,12 +6073,12 @@
           <t>List all available subjects</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -6102,12 +6106,12 @@
           <t>List available grades (10, 11, 12)</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -6115,7 +6119,7 @@
       <c r="G40" s="4" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -6135,7 +6139,7 @@
           <t>Create Connex Pay wallet for user</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -6152,7 +6156,7 @@
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
@@ -6172,7 +6176,7 @@
           <t>P2P money transfer between users</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -6209,7 +6213,7 @@
           <t>Get transaction history</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -8683,7 +8687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9424,12 +9428,12 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>jsonwebtoken</t>
+          <t>bcryptjs</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>^9.x</t>
+          <t>^3.x</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -9439,25 +9443,29 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>JWT creation and verification</t>
+          <t>Legacy-password migration support</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>npm install jsonwebtoken</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr"/>
+          <t>npm install bcryptjs</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Used only to migrate older custom-auth users</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>bcryptjs</t>
+          <t>zod</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>^2.x</t>
+          <t>^3.x</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -9467,29 +9475,25 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Password hashing</t>
+          <t>Request body validation</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>npm install bcryptjs</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Never store plain passwords</t>
-        </is>
-      </c>
+          <t>npm install zod</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>zod</t>
+          <t>ioredis</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>^3.x</t>
+          <t>^5.x</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -9499,12 +9503,12 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Request body validation</t>
+          <t>Redis client for Upstash</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>npm install zod</t>
+          <t>npm install ioredis</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr"/>
@@ -9512,12 +9516,12 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>ioredis</t>
+          <t>node-cron</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>^5.x</t>
+          <t>^3.x</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
@@ -9527,12 +9531,12 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Redis client for Upstash</t>
+          <t>Scheduled jobs (loadshedding refresh)</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>npm install ioredis</t>
+          <t>npm install node-cron</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
@@ -9540,12 +9544,12 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>node-cron</t>
+          <t>axios</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>^3.x</t>
+          <t>^1.x</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -9555,12 +9559,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Scheduled jobs (loadshedding refresh)</t>
+          <t>HTTP client for EskomSePush API</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>npm install node-cron</t>
+          <t>npm install axios</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr"/>
@@ -9568,12 +9572,12 @@
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>axios</t>
+          <t>cors</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>^1.x</t>
+          <t>^2.x</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -9583,12 +9587,12 @@
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>HTTP client for EskomSePush API</t>
+          <t>CORS middleware</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>npm install axios</t>
+          <t>npm install cors</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
@@ -9596,12 +9600,12 @@
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>cors</t>
+          <t>helmet</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>^2.x</t>
+          <t>^8.x</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
@@ -9611,12 +9615,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>CORS middleware</t>
+          <t>Security headers middleware</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>npm install cors</t>
+          <t>npm install helmet</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr"/>
@@ -9624,12 +9628,12 @@
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>helmet</t>
+          <t>express-rate-limit</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>^8.x</t>
+          <t>^7.x</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
@@ -9639,12 +9643,12 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Security headers middleware</t>
+          <t>Rate limiting for auth endpoints</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>npm install helmet</t>
+          <t>npm install express-rate-limit</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
@@ -9652,12 +9656,12 @@
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>express-rate-limit</t>
+          <t>dotenv</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>^7.x</t>
+          <t>^16.x</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
@@ -9667,12 +9671,12 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Rate limiting for auth endpoints</t>
+          <t>Load .env files</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>npm install express-rate-limit</t>
+          <t>npm install dotenv</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr"/>
@@ -9680,12 +9684,12 @@
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>dotenv</t>
+          <t>firebase-admin</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>^16.x</t>
+          <t>^12.x</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -9695,12 +9699,12 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Load .env files</t>
+          <t>Send FCM push notifications</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>npm install dotenv</t>
+          <t>npm install firebase-admin</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
@@ -9708,12 +9712,12 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>firebase-admin</t>
+          <t>multer</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>^12.x</t>
+          <t>^1.x</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -9723,25 +9727,29 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Send FCM push notifications</t>
+          <t>File upload handling</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>npm install firebase-admin</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr"/>
+          <t>npm install multer</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>For image uploads</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>multer</t>
+          <t>uuid</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>^1.x</t>
+          <t>^9.x</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
@@ -9751,47 +9759,15 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>File upload handling</t>
+          <t>Generate UUIDs (if not using Supabase)</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>npm install multer</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>For image uploads</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>uuid</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>^9.x</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Generate UUIDs (if not using Supabase)</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
           <t>npm install uuid</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -9869,22 +9845,22 @@
           <t>0</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Setup &amp; Architecture</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Project init, Supabase setup, GitHub repo, dev environment, folder structure, CI skeleton</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>No revenue — build foundation</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>R0</t>
         </is>
@@ -10038,12 +10014,12 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Connex Logistics</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Ride-hailing (Uber-equivalent, township-first pricing)
 Food delivery (local restaurants + township traders)
@@ -10053,7 +10029,7 @@
 Driver/courier partner app</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Commission per trip/order (15–25%)
 Subscription: Connex Business tier
@@ -10062,7 +10038,7 @@
 White-label logistics API for enterprises</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>R68M/yr at scale</t>
         </is>
@@ -10084,12 +10060,12 @@
           <t>5+</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Connex Enterprise &amp; Expansion</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Multi-country expansion (Zimbabwe, Nigeria, Kenya, Ghana)
 Connex Data &amp; API licensing (anonymised community data)
@@ -10098,7 +10074,7 @@
 SAPS / emergency services SOS integration</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Data licensing
 Government contracts
@@ -10106,7 +10082,7 @@
 Franchise/partner model per country</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>R180M+/yr</t>
         </is>
@@ -10224,7 +10200,7 @@
           <t>Pro: $25/month</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10266,7 +10242,7 @@
           <t>~$10–30/month (scales with usage)</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10295,7 +10271,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>JWT session cache, rate limiting, loadshedding data cache</t>
+          <t>Optional cache, rate limiting, loadshedding data cache</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -10308,19 +10284,19 @@
           <t>Pay-per-use: very cheap</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Optional</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>upstash.com — serverless Redis, works with Railway</t>
+          <t>upstash.com — enable only when in-memory fallback is no longer enough</t>
         </is>
       </c>
     </row>
@@ -10350,7 +10326,7 @@
           <t>Free — no cost for FCM</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10392,7 +10368,7 @@
           <t>Production: $99/month</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10434,7 +10410,7 @@
           <t>Paid tier: R999+/month</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10476,7 +10452,7 @@
           <t>$25 once (no monthly fee)</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10518,7 +10494,7 @@
           <t>$99/year developer account</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10560,7 +10536,7 @@
           <t>$89/month (Plus)</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10812,7 +10788,7 @@
           <t>~$0.0075 per SMS</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10854,7 +10830,7 @@
           <t>Team: $26/month</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -10896,7 +10872,7 @@
           <t>Scale: $450/month</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>